<commit_message>
Test summary 1.1 after re-test: 486 passed, six items closed; figures aligned across the package
</commit_message>
<xml_diff>
--- a/docs/package/out/BrokerVerse_Security_Due_Diligence_Questionnaire.xlsx
+++ b/docs/package/out/BrokerVerse_Security_Due_Diligence_Questionnaire.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Questionnaire'!$A$1:$H$119</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Evidence documents'!$A$1:$B$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Open items'!$A$1:$C$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Open items'!$A$1:$C$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Legend'!$A$1:$B$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1506,9 +1506,9 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>Master &gt; Data Privacy &gt; Consent Register and consent per purpose on the client and prospect (processing, marketing, sharing with insurers), with channel, notice version and evidence. Delivered after the release test of 03 October 2026; re-test of BV-SEC-034 pending [to confirm re-test date]</t>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Master &gt; Data Privacy &gt; Consent Register and consent per purpose on the client and prospect (processing, marketing, sharing with insurers), with channel, notice version and evidence. Delivered after the release test and re-tested on 03 October 2026 (BV-SEC-034 passed)</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1540,9 +1540,9 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>Master &gt; Data Privacy &gt; Data Subject Requests (DSR- numbers), due date 15 calendar days (privacy.request_due_days), personal data export as JSON or Excel. Re-test of BV-SEC-035 pending [to confirm]</t>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Master &gt; Data Privacy &gt; Data Subject Requests (DSR- numbers), due date 15 calendar days (privacy.request_due_days), personal data export as JSON or Excel. Re-tested on 03 October 2026 (BV-SEC-035 passed)</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Housekeeping job removes temporary data on configured periods; audit trail kept by default and never purged below 7 years; business records kept; recommended retention of 10 years for financial and policy records, confirmed by the broker</t>
+          <t>Housekeeping job removes temporary data on configured periods; audit trail kept by default and never purged below 7 years; business records kept; personal data of a client or prospect anonymised on request once privacy.retention_years (10) has passed; recommended retention of 10 years for financial and policy records, confirmed by the broker</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Seven delivered roles; permissions checked by the server on every route (796 of 854 routes need a permission or role, 39 need sign-in only, 19 are public by design); menus deny by default</t>
+          <t>Seven delivered roles; permissions checked by the server on every route (807 of 868 routes need a permission or role, 42 need sign-in only, 19 are public by design); menus deny by default</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3371,19 +3371,19 @@
           <t>What are the patching timelines</t>
         </is>
       </c>
-      <c r="D84" s="3" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E84" s="4" t="inlineStr">
-        <is>
-          <t>Critical patches within [7] days (DPA annex); AIS recommends critical within 14 days and high within 30 days [to confirm one standard]; operating system, PostgreSQL and nginx monthly</t>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Critical security patches within 14 days and high within 30 days; operating system, PostgreSQL and nginx monthly</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>DPA, Annex 2; AIS; PSS, Patching</t>
+          <t>DPA, Annex 2; HSA; AIS; PSS, Patching</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr"/>
@@ -4791,7 +4791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4926,12 +4926,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>One patching standard across DPA and AIS (VUL-02)</t>
+          <t>Philippine hosting partner and support team location (SUB-03, SUB-05)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>iorta TechNXT engineering</t>
+          <t>iorta TechNXT management</t>
         </is>
       </c>
     </row>
@@ -4943,51 +4943,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Philippine hosting partner and support team location (SUB-03, SUB-05)</t>
+          <t>IC circular numbers and IC examination right (REG-01, REG-03, AUD-03)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>iorta TechNXT management</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>IC circular numbers and IC examination right (REG-01, REG-03, AUD-03)</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
           <t>Broker compliance officer with iorta TechNXT legal</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Re-test of the data privacy cases BV-SEC-034 and BV-SEC-035 (DPA-05, DPA-06)</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>iorta TechNXT QA</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C11"/>
+  <autoFilter ref="A1:C9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>